<commit_message>
Separate costs and effects in recipes
</commit_message>
<xml_diff>
--- a/tabella_gioco_A3_ricostruita.xlsx
+++ b/tabella_gioco_A3_ricostruita.xlsx
@@ -521,8 +521,8 @@
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>CIABATTA
-U↪ : 3 esagoni in ogni direzione
-3U▽: schiva</t>
+Effetto: U↪ 3 esagoni in ogni direzione
+Effetto: 3U▽ schiva</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -532,17 +532,15 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>1 bacca
-1 RAMO
-Accessorio: NO</t>
+          <t>Costo - bacca x1, ramo x1
+Prerequisito - accessorio no</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1 PELLE  
-1 BACCA
-U ↪ movimento 4
-1 movimento non azione a round</t>
+          <t>Costo: pelle:1; bacca:1
+Effetto: U↪ movimento 4
+Regola: 1 movimento non azione a round</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -550,9 +548,8 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>1 Succo di bacca
-1 LASTRA potenziata
-U⚔: 1 danno e allontana 1</t>
+          <t>Costo: succo_di_bacca:1; lastra_potenziata:1
+Effetto: U⚔ 1 danno e allontana 1</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -560,8 +557,8 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>2 bacche
-U↪: salta 3</t>
+          <t>Costo: bacca:2
+Effetto: U↪ salta 3</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
@@ -573,8 +570,8 @@
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>LASTRA
-U⚔: 2 danni
-U✱: distrarre</t>
+Effetto: U⚔ 2 danni
+Effetto: U✱ distrarre</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -584,16 +581,15 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>1 PIETRA
-Accessorio: pietra, attrezzo</t>
+          <t>Costo - pietra x1
+Prerequisito - accessorio pietra, attrezzo</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>1 utilizzo attrezzo 
-1 utilizzo lastra  
-perde abilità
-U⚔:3 danni a scalare E5</t>
+          <t>Costo: utilizzo_attrezzo:1; utilizzo_lastra:1
+Regola: perde abilità
+Effetto: U⚔ 3 danni a scalare E5</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -603,8 +599,8 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>1 utilizzo attrezzo
-U⚔: 1 danno G 6</t>
+          <t>Costo: utilizzo_attrezzo:1
+Effetto: U⚔ 1 danno G 6</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -624,8 +620,8 @@
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>COLTELLO
-U ⚔: 2 danni
-U O: estrai 1, ottieni 2</t>
+Effetto: U⚔ 2 danni
+Effetto: UO estrai 1, ottieni 2</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -635,16 +631,15 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>1 PIETRA
-Accessorio: pietra, attrezzo</t>
+          <t>Costo - pietra x1
+Prerequisito - accessorio pietra, attrezzo</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>1 utilizzo attrezzo 
-1 utilizzo lastra 
-perde abilità
-U⚔: 1danno  e ferisci</t>
+          <t>Costo: utilizzo_attrezzo:1; utilizzo_lastra:1
+Regola: perde abilità
+Effetto: U⚔ 1 danno e ferisci</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -654,9 +649,8 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>1 utilizzo attrezzo 
-1 PIETRA
-U⚔: 2 danni G 3</t>
+          <t>Costo: utilizzo_attrezzo:1; pietra:1
+Effetto: U⚔ 2 danni G 3</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -664,7 +658,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>PELLE</t>
+          <t>Costo: pelle:1</t>
         </is>
       </c>
       <c r="I4" s="3" t="n">
@@ -676,9 +670,9 @@
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>BASTONE
-U⚔: 2 danni in R
-U↪: 4 esagoni in linea retta
-U▽: para 1</t>
+Effetto: U⚔ 2 danni in R
+Effetto: U↪ 4 esagoni in linea retta
+Effetto: U▽ para 1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -688,14 +682,14 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>1 RAMO
-Accessorio: coltello, attrezzo</t>
+          <t>Costo - ramo x1
+Prerequisito - accessorio coltello, attrezzo</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>1 utilizzo coltello
-U⚔: 2 danni G 4</t>
+          <t>Costo: utilizzo_coltello:1
+Effetto: U⚔ 2 danni G 4</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -705,10 +699,9 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>1 PELLE
-1 succo di bacca
-U⚔: 3 danni
-U▽: difendi 3</t>
+          <t>Costo: pelle:1; succo_di_bacca:1
+Effetto: U⚔ 3 danni
+Effetto: U▽ difendi 3</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -718,10 +711,9 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Accessorio: coltello
-Accessorio: succo di bacca
-1 RAMO
-U↪: muovi 1, poi 5 linee retta</t>
+          <t>Costo: ramo:1
+Prerequisito: accessorio coltello, succo di bacca
+Effetto: U↪ muovi 1, poi 5 linee retta</t>
         </is>
       </c>
       <c r="I5" s="3" t="n"/>
@@ -731,8 +723,8 @@
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>ATTREZZO
-U⚔: 3 danni
-U O: estrai fino a 3 anelli</t>
+Effetto: U⚔ 3 danni
+Effetto: UO estrai fino a 3 anelli</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -742,16 +734,15 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>1 RAMO
-1 PIETRA
-Accessorio: pietra, attrezzo</t>
+          <t>Costo - ramo x1, pietra x1
+Prerequisito - accessorio pietra, attrezzo</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Accessorio: LASTRA
-un azione aggiuntiva
-U⚔: 3 danni G 3</t>
+          <t>Prerequisito: accessorio lastra
+Regola: un azione aggiuntiva
+Effetto: U⚔ 3 danni G 3</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -761,10 +752,8 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 1Succo di bacca
- 1 PELLE
-U⚔: 4 danni  L3
-                       </t>
+          <t>Costo: succo_di_bacca:1; pelle:1
+Effetto: U⚔ 4 danni L3</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -774,9 +763,8 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>BASTONE
-Succo di bacca
-2U O: estrai 1, ottieni 3</t>
+          <t>Costo: bastone:1; succo_di_bacca:1
+Effetto: 2UO estrai 1, ottieni 3</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -790,10 +778,10 @@
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>TORCIA
--accendi(illumina raggio 1)
--spegni
-U✱: infila a terra
-2U▽:evita un attacco</t>
+Effetto: accendi illumina raggio 1
+Effetto: spegni
+Effetto: U✱ infila a terra
+Effetto: 2U▽ evita un attacco</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -803,18 +791,16 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>1 RAMO
-1 PIETRA
-1 BACCA</t>
+          <t>Costo - ramo x1, pietra x1, bacca x1</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>1 Succo di bacca
--accendi(illumina raggio 2)
--spegni
-4U⚔:brucia
-4 U▽: evita e brucia</t>
+          <t>Costo: succo_di_bacca:1
+Effetto: accendi illumina raggio 2
+Effetto: spegni
+Effetto: 4U⚔ brucia
+Effetto: 4U▽ evita e brucia</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -844,7 +830,6 @@
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
-    <row r="9"/>
     <row r="10" ht="27.75" customHeight="1" s="12">
       <c r="A10" s="13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Improve recipe text spacing
</commit_message>
<xml_diff>
--- a/tabella_gioco_A3_ricostruita.xlsx
+++ b/tabella_gioco_A3_ricostruita.xlsx
@@ -521,8 +521,8 @@
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>CIABATTA
-Effetto: U↪ 3 esagoni in ogni direzione
-Effetto: 3U▽ schiva</t>
+Effetto - U↪ 3 esagoni in ogni direzione
+Effetto - 3U▽ schiva</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -532,15 +532,15 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Costo - bacca x1, ramo x1
-Prerequisito - accessorio no</t>
+          <t>Costo - 1 bacca, 1 ramo
+Prerequisito - nessun requisito</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Costo: pelle:1; bacca:1
-Effetto: U↪ movimento 4
-Regola: 1 movimento non azione a round</t>
+          <t>Costo - 1 pelle, 1 bacca
+Effetto - U↪ movimento 4
+Regola - 1 movimento non azione per round</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
@@ -548,8 +548,8 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Costo: succo_di_bacca:1; lastra_potenziata:1
-Effetto: U⚔ 1 danno e allontana 1</t>
+          <t>Costo - 1 succo di bacca, 1 lastra potenziata
+Effetto - U⚔ 1 danno e allontana 1</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -557,8 +557,8 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Costo: bacca:2
-Effetto: U↪ salta 3</t>
+          <t>Costo - 2 bacche
+Effetto - U↪ salta 3</t>
         </is>
       </c>
       <c r="I2" s="3" t="n">
@@ -570,8 +570,8 @@
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>LASTRA
-Effetto: U⚔ 2 danni
-Effetto: U✱ distrarre</t>
+Effetto - U⚔ 2 danni
+Effetto - U✱ distrarre</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -581,15 +581,15 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Costo - pietra x1
+          <t>Costo - 1 pietra
 Prerequisito - accessorio pietra, attrezzo</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Costo: utilizzo_attrezzo:1; utilizzo_lastra:1
-Regola: perde abilità
-Effetto: U⚔ 3 danni a scalare E5</t>
+          <t>Costo - 1 utilizzo attrezzo, 1 utilizzo lastra
+Regola - perde abilità
+Effetto - U⚔ 3 danni a scalare E5</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -599,8 +599,8 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Costo: utilizzo_attrezzo:1
-Effetto: U⚔ 1 danno G 6</t>
+          <t>Costo - 1 utilizzo attrezzo
+Effetto - U⚔ 1 danno G 6</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -620,8 +620,8 @@
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>COLTELLO
-Effetto: U⚔ 2 danni
-Effetto: UO estrai 1, ottieni 2</t>
+Effetto - U⚔ 2 danni
+Effetto - U O estrai 1, ottieni 2</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -631,15 +631,15 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Costo - pietra x1
+          <t>Costo - 1 pietra
 Prerequisito - accessorio pietra, attrezzo</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Costo: utilizzo_attrezzo:1; utilizzo_lastra:1
-Regola: perde abilità
-Effetto: U⚔ 1 danno e ferisci</t>
+          <t>Costo - 1 utilizzo attrezzo, 1 utilizzo lastra
+Regola - perde abilità
+Effetto - U⚔ 1 danno e ferisci</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -649,8 +649,8 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Costo: utilizzo_attrezzo:1; pietra:1
-Effetto: U⚔ 2 danni G 3</t>
+          <t>Costo - 1 utilizzo attrezzo, 1 pietra
+Effetto - U⚔ 2 danni G 3</t>
         </is>
       </c>
       <c r="G4" s="3" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Costo: pelle:1</t>
+          <t>Costo - 1 pelle</t>
         </is>
       </c>
       <c r="I4" s="3" t="n">
@@ -670,9 +670,9 @@
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>BASTONE
-Effetto: U⚔ 2 danni in R
-Effetto: U↪ 4 esagoni in linea retta
-Effetto: U▽ para 1</t>
+Effetto - U⚔ 2 danni in R
+Effetto - U↪ 4 esagoni in linea retta
+Effetto - U▽ para 1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -682,14 +682,14 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Costo - ramo x1
+          <t>Costo - 1 ramo
 Prerequisito - accessorio coltello, attrezzo</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Costo: utilizzo_coltello:1
-Effetto: U⚔ 2 danni G 4</t>
+          <t>Costo - 1 utilizzo coltello
+Effetto - U⚔ 2 danni G 4</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -699,9 +699,9 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Costo: pelle:1; succo_di_bacca:1
-Effetto: U⚔ 3 danni
-Effetto: U▽ difendi 3</t>
+          <t>Costo - 1 pelle, 1 succo di bacca
+Effetto - U⚔ 3 danni
+Effetto - U▽ difendi 3</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -711,9 +711,9 @@
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Costo: ramo:1
-Prerequisito: accessorio coltello, succo di bacca
-Effetto: U↪ muovi 1, poi 5 linee retta</t>
+          <t>Costo - 1 ramo
+Prerequisito - accessorio coltello, succo di bacca
+Effetto - U↪ muovi 1, poi 5 in linea retta</t>
         </is>
       </c>
       <c r="I5" s="3" t="n"/>
@@ -723,8 +723,8 @@
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>ATTREZZO
-Effetto: U⚔ 3 danni
-Effetto: UO estrai fino a 3 anelli</t>
+Effetto - U⚔ 3 danni
+Effetto - U O estrai fino a 3 anelli</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -734,15 +734,15 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Costo - ramo x1, pietra x1
+          <t>Costo - 1 ramo, 1 pietra
 Prerequisito - accessorio pietra, attrezzo</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Prerequisito: accessorio lastra
-Regola: un azione aggiuntiva
-Effetto: U⚔ 3 danni G 3</t>
+          <t>Prerequisito - accessorio lastra
+Regola - un'azione aggiuntiva
+Effetto - U⚔ 3 danni G 3</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -752,8 +752,8 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Costo: succo_di_bacca:1; pelle:1
-Effetto: U⚔ 4 danni L3</t>
+          <t>Costo - 1 succo di bacca, 1 pelle
+Effetto - U⚔ 4 danni L3</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -763,8 +763,8 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Costo: bastone:1; succo_di_bacca:1
-Effetto: 2UO estrai 1, ottieni 3</t>
+          <t>Costo - 1 bastone, 1 succo di bacca
+Effetto - 2U O estrai 1, ottieni 3</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -778,10 +778,10 @@
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>TORCIA
-Effetto: accendi illumina raggio 1
-Effetto: spegni
-Effetto: U✱ infila a terra
-Effetto: 2U▽ evita un attacco</t>
+Effetto - accendi: illumina raggio 1
+Effetto - spegni
+Effetto - U✱ infila a terra
+Effetto - 2U▽ evita un attacco</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -791,16 +791,16 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Costo - ramo x1, pietra x1, bacca x1</t>
+          <t>Costo - 1 ramo, 1 pietra, 1 bacca</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Costo: succo_di_bacca:1
-Effetto: accendi illumina raggio 2
-Effetto: spegni
-Effetto: 4U⚔ brucia
-Effetto: 4U▽ evita e brucia</t>
+          <t>Costo - 1 succo di bacca
+Effetto - accendi: illumina raggio 2
+Effetto - spegni
+Effetto - 4U⚔ brucia
+Effetto - 4U▽ evita e brucia</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">

</xml_diff>